<commit_message>
Update Amkor credit model with break-even sheet
</commit_message>
<xml_diff>
--- a/files/Amkor_Credit_Analysis_Eisen_Hy.xlsx
+++ b/files/Amkor_Credit_Analysis_Eisen_Hy.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit Summary" sheetId="1" r:id="R73bf8b7bc2cf44d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R29feb9eaaf2c42d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="Rbaff6abf0f4542e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt Schedule" sheetId="4" r:id="R9ea0ddc53c704ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials" sheetId="5" r:id="Ref5069e5cfd9499b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Spread" sheetId="6" r:id="R68f909d5a083425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="7" r:id="R325ea9451234483b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit Summary" sheetId="1" r:id="R626af04070a847e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R47783f65a3d6487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R1995158ca7f04196"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt Schedule" sheetId="4" r:id="Rb7b3c3f3549049b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials" sheetId="5" r:id="R0471006fab174991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Spread" sheetId="6" r:id="Rdbeb1eda962141c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="7" r:id="R601f3bf1d8214503"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit Break-even" sheetId="8" r:id="Rbdf450c312444357"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,654 +19,892 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="12">
-    <x:numFmt numFmtId="200" formatCode="#,##0.0;(#,##0.0);&quot;—&quot;"/>
-    <x:numFmt numFmtId="201" formatCode="#,##0"/>
-    <x:numFmt numFmtId="202" formatCode="#,##0;(#,##0);&quot;—&quot;"/>
-    <x:numFmt numFmtId="203" formatCode="@"/>
-    <x:numFmt numFmtId="204" formatCode="0.0%;(0.0%);&quot;—&quot;"/>
-    <x:numFmt numFmtId="205" formatCode="0"/>
-    <x:numFmt numFmtId="206" formatCode="  @"/>
-    <x:numFmt numFmtId="207" formatCode="$#,##0.0;($#,##0.0);&quot;—&quot;"/>
-    <x:numFmt numFmtId="208" formatCode="0.00&quot;x&quot;;(0.00&quot;x&quot;);&quot;—&quot;"/>
-    <x:numFmt numFmtId="209" formatCode="0.0&quot; days&quot;"/>
-    <x:numFmt numFmtId="210" formatCode="0.0"/>
-    <x:numFmt numFmtId="211" formatCode="[&gt;=0.005]0.00;[&lt;=-0.005](0.00);0.00"/>
-  </x:numFmts>
-  <x:fonts count="20">
-    <x:font>
-      <x:sz val="11"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF182C3A"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="20"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF647783"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF137447"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF0056B3"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF0056B3"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:sz val="9"/>
-      <x:color rgb="FF137447"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF182C3A"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF137447"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:i/>
-      <x:sz val="11"/>
-      <x:color rgb="FF182C3A"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:i/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:i/>
-      <x:sz val="11"/>
-      <x:color rgb="FF137447"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="14"/>
-      <x:color rgb="FF182C3A"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF647783"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FF182C3A"/>
-      <x:name val="Aptos"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="6">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF15364A"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF3CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF147D92"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE9F3F6"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="2">
-    <x:border/>
-    <x:border>
-      <x:top style="thin">
-        <x:color rgb="FF9AB0BC"/>
-      </x:top>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </x:cellStyleXfs>
-  <x:cellXfs count="131">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="202" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="203" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="203" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="203" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="204" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="208" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="209" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="209" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="203" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="203" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="209" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="208" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="208" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="208" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="210" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="210" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="204" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="204" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="205" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="210" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="17" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="17" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="208" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="203" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="203" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="207" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="211" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="211" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="211" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="211" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0"/>
-  </x:cellStyles>
-  <x:dxfs count="15">
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA32626"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDEBEC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF137447"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE6F3EC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF137447"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE6F3EC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF137447"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE6F3EC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF137447"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE6F3EC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-  </x:dxfs>
-</x:styleSheet>
+<ns0:styleSheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:numFmts count="14">
+    <ns0:numFmt numFmtId="200" formatCode="#,##0.0;(#,##0.0);&quot;—&quot;"/>
+    <ns0:numFmt numFmtId="201" formatCode="#,##0"/>
+    <ns0:numFmt numFmtId="202" formatCode="#,##0;(#,##0);&quot;—&quot;"/>
+    <ns0:numFmt numFmtId="203" formatCode="@"/>
+    <ns0:numFmt numFmtId="204" formatCode="0.0%;(0.0%);&quot;—&quot;"/>
+    <ns0:numFmt numFmtId="205" formatCode="0"/>
+    <ns0:numFmt numFmtId="206" formatCode="  @"/>
+    <ns0:numFmt numFmtId="207" formatCode="$#,##0.0;($#,##0.0);&quot;—&quot;"/>
+    <ns0:numFmt numFmtId="208" formatCode="0.00&quot;x&quot;;(0.00&quot;x&quot;);&quot;—&quot;"/>
+    <ns0:numFmt numFmtId="209" formatCode="0.0&quot; days&quot;"/>
+    <ns0:numFmt numFmtId="210" formatCode="0.0"/>
+    <ns0:numFmt numFmtId="211" formatCode="[&gt;=0.005]0.00;[&lt;=-0.005](0.00);0.00"/>
+    <ns0:numFmt numFmtId="212" formatCode="#,##0.0;(#,##0.0);&quot;–&quot;"/>
+    <ns0:numFmt numFmtId="213" formatCode="0.0%;(0.0%);&quot;–&quot;"/>
+  </ns0:numFmts>
+  <ns0:fonts count="30">
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:name val="Carlito"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF182C3A"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="20"/>
+      <ns0:color rgb="FFFFFFFF"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="10"/>
+      <ns0:color rgb="FF647783"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF137447"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="10"/>
+      <ns0:color rgb="FF0056B3"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FFFFFFFF"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF0056B3"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="9"/>
+      <ns0:color rgb="FF137447"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF000000"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF182C3A"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF137447"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF000000"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:i/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF182C3A"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:i/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF000000"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:i/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF137447"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="10"/>
+      <ns0:color rgb="FF000000"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="14"/>
+      <ns0:color rgb="FF182C3A"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF647783"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="10"/>
+      <ns0:color rgb="FF182C3A"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF172B4D"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="16"/>
+      <ns0:color rgb="FF234F78"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:i/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF58677A"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF00804A"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF58677A"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF234F78"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:i/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF172B4D"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF172B4D"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:i/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF172B4D"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="10"/>
+      <ns0:color rgb="FF58677A"/>
+      <ns0:name val="Aptos"/>
+    </ns0:font>
+  </ns0:fonts>
+  <ns0:fills count="8">
+    <ns0:fill>
+      <ns0:patternFill patternType="none"/>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="gray125"/>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FF15364A"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFFFF3CC"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FF147D92"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFE9F3F6"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FF234F78"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFDFEAF3"/>
+      </ns0:patternFill>
+    </ns0:fill>
+  </ns0:fills>
+  <ns0:borders count="7">
+    <ns0:border/>
+    <ns0:border>
+      <ns0:top style="thin">
+        <ns0:color rgb="FF9AB0BC"/>
+      </ns0:top>
+    </ns0:border>
+    <ns0:border>
+      <ns0:bottom style="thin">
+        <ns0:color rgb="FF234F78"/>
+      </ns0:bottom>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="dotted">
+        <ns0:color rgb="FF234F78"/>
+      </ns0:left>
+      <ns0:top style="dotted">
+        <ns0:color rgb="FF234F78"/>
+      </ns0:top>
+      <ns0:bottom style="dotted">
+        <ns0:color rgb="FF234F78"/>
+      </ns0:bottom>
+    </ns0:border>
+    <ns0:border>
+      <ns0:top style="dotted">
+        <ns0:color rgb="FF234F78"/>
+      </ns0:top>
+      <ns0:bottom style="dotted">
+        <ns0:color rgb="FF234F78"/>
+      </ns0:bottom>
+    </ns0:border>
+    <ns0:border>
+      <ns0:right style="dotted">
+        <ns0:color rgb="FF234F78"/>
+      </ns0:right>
+      <ns0:top style="dotted">
+        <ns0:color rgb="FF234F78"/>
+      </ns0:top>
+      <ns0:bottom style="dotted">
+        <ns0:color rgb="FF234F78"/>
+      </ns0:bottom>
+    </ns0:border>
+    <ns0:border>
+      <ns0:top style="thin">
+        <ns0:color rgb="FFCAD4DD"/>
+      </ns0:top>
+    </ns0:border>
+  </ns0:borders>
+  <ns0:cellStyleXfs count="1">
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </ns0:cellStyleXfs>
+  <ns0:cellXfs count="167">
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="201" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="201" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="202" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="202" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="203" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="203" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="203" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="201" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="201" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="204" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="204" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="204" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="204" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="207" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="204" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="204" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="204" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="208" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="209" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="209" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="203" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="203" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="205" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="204" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="204" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="209" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="205" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="205" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="204" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="208" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="208" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="208" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="210" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="210" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="207" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="207" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="204" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="204" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="205" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="210" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="200" fontId="17" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="17" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="208" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="203" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="203" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="207" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="211" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="211" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="211" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="211" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="200" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="20" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="212" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="212" fontId="25" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="213" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="213" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="213" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="213" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="212" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="27" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="212" fontId="27" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="213" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="213" fontId="28" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment vertical="center" wrapText="1"/>
+    </ns0:xf>
+  </ns0:cellXfs>
+  <ns0:cellStyles count="1">
+    <ns0:cellStyle name="Normal" xfId="0"/>
+  </ns0:cellStyles>
+  <ns0:dxfs count="17">
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32626"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:color rgb="FF137447"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFE6F3EC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:color rgb="FF137447"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFE6F3EC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:color rgb="FF137447"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFE6F3EC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:color rgb="FF137447"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFE6F3EC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32832"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:font>
+        <ns0:b/>
+        <ns0:color rgb="FFA32832"/>
+      </ns0:font>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFFDEBEC"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+  </ns0:dxfs>
+</ns0:styleSheet>
 </file>
 
 <file path=xl/drawings/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1049,7 +1288,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2525848d0a8b4a3b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9ae64f59ceab43f7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1084,7 +1323,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re8064b5df06d4a3f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9148a473ab2a47a7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2317,7 +2556,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddae3de843d44d05"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90690df033b445a"/>
 </x:worksheet>
 </file>
 
@@ -7800,7 +8039,7 @@
     <x:mergeCell ref="C57:J57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1396ba6826184d1c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc14130684c204eb2"/>
 </x:worksheet>
 </file>
 
@@ -13839,4 +14078,625 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF234F78"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="3" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="3" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="59" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2" ht="29" customHeight="1">
+      <x:c r="C2" s="134" t="str">
+        <x:v>AMKOR CREDIT BREAK-EVEN</x:v>
+      </x:c>
+      <x:c r="D2" s="134"/>
+      <x:c r="E2" s="134"/>
+      <x:c r="F2" s="134"/>
+      <x:c r="G2" s="134"/>
+    </x:row>
+    <x:row r="3" ht="23" customHeight="1">
+      <x:c r="C3" s="135" t="str">
+        <x:v>USD millions. Period-end liquidity test.</x:v>
+      </x:c>
+      <x:c r="D3" s="135"/>
+      <x:c r="E3" s="135"/>
+      <x:c r="F3" s="135"/>
+      <x:c r="G3" s="135"/>
+    </x:row>
+    <x:row r="4" ht="23" customHeight="1">
+      <x:c r="C4" s="132" t="str">
+        <x:v>Case selected:</x:v>
+      </x:c>
+      <x:c r="D4" s="140" t="str">
+        <x:f>'Assumptions'!D7</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="E4" s="141"/>
+      <x:c r="F4" s="142"/>
+      <x:c r="G4" s="132"/>
+    </x:row>
+    <x:row r="5" ht="23" customHeight="1">
+      <x:c r="C5" s="143" t="str">
+        <x:v>Change the case using Assumptions!D7. Both alternatives below update automatically.</x:v>
+      </x:c>
+      <x:c r="D5" s="143"/>
+      <x:c r="E5" s="143"/>
+      <x:c r="F5" s="143"/>
+      <x:c r="G5" s="143"/>
+    </x:row>
+    <x:row r="6" ht="23" customHeight="1">
+      <x:c r="C6" s="132"/>
+      <x:c r="D6" s="132"/>
+      <x:c r="E6" s="132"/>
+      <x:c r="F6" s="132"/>
+      <x:c r="G6" s="132"/>
+    </x:row>
+    <x:row r="7" ht="27" customHeight="1">
+      <x:c r="C7" s="146" t="str">
+        <x:v>Liquidity and spending</x:v>
+      </x:c>
+      <x:c r="D7" s="146" t="str">
+        <x:v>2026 H2E</x:v>
+      </x:c>
+      <x:c r="E7" s="146" t="str">
+        <x:v>2027E</x:v>
+      </x:c>
+      <x:c r="F7" s="146" t="str">
+        <x:v>2028E</x:v>
+      </x:c>
+      <x:c r="G7" s="146" t="str">
+        <x:v>2029E</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="23" customHeight="1">
+      <x:c r="C8" s="132" t="str">
+        <x:v>Modeled closing liquidity before remedies</x:v>
+      </x:c>
+      <x:c r="D8" s="149" t="n">
+        <x:f>'Forecast'!D59</x:f>
+        <x:v>931.6386302362209</x:v>
+      </x:c>
+      <x:c r="E8" s="149" t="n">
+        <x:f>'Forecast'!E59</x:f>
+        <x:v>688.3566673074747</x:v>
+      </x:c>
+      <x:c r="F8" s="149" t="n">
+        <x:f>'Forecast'!F59</x:f>
+        <x:v>-1544.5139335999293</x:v>
+      </x:c>
+      <x:c r="G8" s="149" t="n">
+        <x:f>'Forecast'!G59</x:f>
+        <x:v>-2515.4906200948335</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="23" customHeight="1">
+      <x:c r="C9" s="132" t="str">
+        <x:v>Minimum liquidity reserve</x:v>
+      </x:c>
+      <x:c r="D9" s="149" t="n">
+        <x:f>'Forecast'!D60</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="E9" s="149" t="n">
+        <x:f>'Forecast'!E60</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="F9" s="149" t="n">
+        <x:f>'Forecast'!F60</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G9" s="149" t="n">
+        <x:f>'Forecast'!G60</x:f>
+        <x:v>500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="23" customHeight="1">
+      <x:c r="C10" s="158" t="str">
+        <x:v>Liquidity headroom / (shortfall)</x:v>
+      </x:c>
+      <x:c r="D10" s="159" t="n">
+        <x:f>D8-D9</x:f>
+        <x:v>431.63863023622093</x:v>
+      </x:c>
+      <x:c r="E10" s="159" t="n">
+        <x:f>E8-E9</x:f>
+        <x:v>188.3566673074747</x:v>
+      </x:c>
+      <x:c r="F10" s="159" t="n">
+        <x:f>F8-F9</x:f>
+        <x:v>-2044.5139335999293</x:v>
+      </x:c>
+      <x:c r="G10" s="159" t="n">
+        <x:f>G8-G9</x:f>
+        <x:v>-3015.4906200948335</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="23" customHeight="1">
+      <x:c r="C11" s="132" t="str">
+        <x:v>Planned cash capital expenditures</x:v>
+      </x:c>
+      <x:c r="D11" s="149" t="n">
+        <x:f>'Forecast'!D49</x:f>
+        <x:v>2061.575</x:v>
+      </x:c>
+      <x:c r="E11" s="149" t="n">
+        <x:f>'Forecast'!E49</x:f>
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="F11" s="149" t="n">
+        <x:f>'Forecast'!F49</x:f>
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="G11" s="149" t="n">
+        <x:f>'Forecast'!G49</x:f>
+        <x:v>1500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="23" customHeight="1">
+      <x:c r="C12" s="132" t="str">
+        <x:v>Protected maintenance capex estimate</x:v>
+      </x:c>
+      <x:c r="D12" s="149" t="n">
+        <x:f>D11*'Assumptions'!$D$57</x:f>
+        <x:v>618.4725</x:v>
+      </x:c>
+      <x:c r="E12" s="149" t="n">
+        <x:f>E11*'Assumptions'!$D$57</x:f>
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="F12" s="149" t="n">
+        <x:f>F11*'Assumptions'!$D$57</x:f>
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="G12" s="149" t="n">
+        <x:f>G11*'Assumptions'!$D$57</x:f>
+        <x:v>450</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="23" customHeight="1">
+      <x:c r="C13" s="132" t="str">
+        <x:v>Discretionary capex available to defer</x:v>
+      </x:c>
+      <x:c r="D13" s="149" t="n">
+        <x:f>MAX(0,D11-D12)</x:f>
+        <x:v>1443.1025</x:v>
+      </x:c>
+      <x:c r="E13" s="149" t="n">
+        <x:f>MAX(0,E11-E12)</x:f>
+        <x:v>2100</x:v>
+      </x:c>
+      <x:c r="F13" s="149" t="n">
+        <x:f>MAX(0,F11-F12)</x:f>
+        <x:v>1750</x:v>
+      </x:c>
+      <x:c r="G13" s="149" t="n">
+        <x:f>MAX(0,G11-G12)</x:f>
+        <x:v>1050</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="23" customHeight="1">
+      <x:c r="C14" s="132" t="str">
+        <x:v>Cumulative planned cash capex</x:v>
+      </x:c>
+      <x:c r="D14" s="149" t="n">
+        <x:f>SUM($D11:D11)</x:f>
+        <x:v>2061.575</x:v>
+      </x:c>
+      <x:c r="E14" s="149" t="n">
+        <x:f>SUM($D11:E11)</x:f>
+        <x:v>5061.575</x:v>
+      </x:c>
+      <x:c r="F14" s="149" t="n">
+        <x:f>SUM($D11:F11)</x:f>
+        <x:v>7561.575</x:v>
+      </x:c>
+      <x:c r="G14" s="149" t="n">
+        <x:f>SUM($D11:G11)</x:f>
+        <x:v>9061.575</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="C15" s="148" t="str">
+        <x:v>ALTERNATIVE A: FUND PLANNED CAPEX</x:v>
+      </x:c>
+      <x:c r="D15" s="150"/>
+      <x:c r="E15" s="150"/>
+      <x:c r="F15" s="150"/>
+      <x:c r="G15" s="150"/>
+    </x:row>
+    <x:row r="16" ht="23" customHeight="1">
+      <x:c r="C16" s="158" t="str">
+        <x:v>Cumulative funding committed by period-end</x:v>
+      </x:c>
+      <x:c r="D16" s="159" t="n">
+        <x:f>MAX(0,D9-D8)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="159" t="n">
+        <x:f>MAX(D16,E9-E8)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="159" t="n">
+        <x:f>MAX(E16,F9-F8)</x:f>
+        <x:v>2044.5139335999293</x:v>
+      </x:c>
+      <x:c r="G16" s="159" t="n">
+        <x:f>MAX(F16,G9-G8)</x:f>
+        <x:v>3015.4906200948335</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="23" customHeight="1">
+      <x:c r="C17" s="158" t="str">
+        <x:v>Additional funding first needed this period</x:v>
+      </x:c>
+      <x:c r="D17" s="159" t="n">
+        <x:f>D16</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="159" t="n">
+        <x:f>E16-D16</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="159" t="n">
+        <x:f>F16-E16</x:f>
+        <x:v>2044.5139335999293</x:v>
+      </x:c>
+      <x:c r="G17" s="159" t="n">
+        <x:f>G16-F16</x:f>
+        <x:v>970.9766864949042</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="23" customHeight="1">
+      <x:c r="C18" s="158" t="str">
+        <x:v>Closing liquidity with funding</x:v>
+      </x:c>
+      <x:c r="D18" s="159" t="n">
+        <x:f>D8+D16</x:f>
+        <x:v>931.6386302362209</x:v>
+      </x:c>
+      <x:c r="E18" s="159" t="n">
+        <x:f>E8+E16</x:f>
+        <x:v>688.3566673074747</x:v>
+      </x:c>
+      <x:c r="F18" s="159" t="n">
+        <x:f>F8+F16</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G18" s="159" t="n">
+        <x:f>G8+G16</x:f>
+        <x:v>500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="23" customHeight="1">
+      <x:c r="C19" s="132"/>
+      <x:c r="D19" s="149"/>
+      <x:c r="E19" s="149"/>
+      <x:c r="F19" s="149"/>
+      <x:c r="G19" s="149"/>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="C20" s="148" t="str">
+        <x:v>ALTERNATIVE B: DEFER DISCRETIONARY CAPEX FIRST</x:v>
+      </x:c>
+      <x:c r="D20" s="150"/>
+      <x:c r="E20" s="150"/>
+      <x:c r="F20" s="150"/>
+      <x:c r="G20" s="150"/>
+    </x:row>
+    <x:row r="21" ht="23" customHeight="1">
+      <x:c r="C21" s="162" t="str">
+        <x:v>Minimum uniform capex cut needed across horizon</x:v>
+      </x:c>
+      <x:c r="D21" s="163" t="n">
+        <x:f>IF(COUNT(D29:G29)=4,MAX(D29:G29),"n.a.")</x:f>
+        <x:v>0.3327777588437808</x:v>
+      </x:c>
+      <x:c r="E21" s="163"/>
+      <x:c r="F21" s="163"/>
+      <x:c r="G21" s="163"/>
+    </x:row>
+    <x:row r="22" ht="23" customHeight="1">
+      <x:c r="C22" s="132" t="str">
+        <x:v>Capex cash savings this period (maintenance protected)</x:v>
+      </x:c>
+      <x:c r="D22" s="149" t="n">
+        <x:f>MIN(D13,D11*$D$21)</x:f>
+        <x:v>686.0463081883673</x:v>
+      </x:c>
+      <x:c r="E22" s="149" t="n">
+        <x:f>MIN(E13,E11*$D$21)</x:f>
+        <x:v>998.3332765313424</x:v>
+      </x:c>
+      <x:c r="F22" s="149" t="n">
+        <x:f>MIN(F13,F11*$D$21)</x:f>
+        <x:v>831.944397109452</x:v>
+      </x:c>
+      <x:c r="G22" s="149" t="n">
+        <x:f>MIN(G13,G11*$D$21)</x:f>
+        <x:v>499.1666382656712</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="23" customHeight="1">
+      <x:c r="C23" s="132" t="str">
+        <x:v>Cumulative capex cash savings</x:v>
+      </x:c>
+      <x:c r="D23" s="149" t="n">
+        <x:f>D22</x:f>
+        <x:v>686.0463081883673</x:v>
+      </x:c>
+      <x:c r="E23" s="149" t="n">
+        <x:f>SUM(D23,E22)</x:f>
+        <x:v>1684.3795847197098</x:v>
+      </x:c>
+      <x:c r="F23" s="149" t="n">
+        <x:f>SUM(E23,F22)</x:f>
+        <x:v>2516.3239818291618</x:v>
+      </x:c>
+      <x:c r="G23" s="149" t="n">
+        <x:f>SUM(F23,G22)</x:f>
+        <x:v>3015.490620094833</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="23" customHeight="1">
+      <x:c r="C24" s="158" t="str">
+        <x:v>Remaining period cash capex</x:v>
+      </x:c>
+      <x:c r="D24" s="159" t="n">
+        <x:f>D11-D22</x:f>
+        <x:v>1375.5286918116326</x:v>
+      </x:c>
+      <x:c r="E24" s="159" t="n">
+        <x:f>E11-E22</x:f>
+        <x:v>2001.6667234686574</x:v>
+      </x:c>
+      <x:c r="F24" s="159" t="n">
+        <x:f>F11-F22</x:f>
+        <x:v>1668.055602890548</x:v>
+      </x:c>
+      <x:c r="G24" s="159" t="n">
+        <x:f>G11-G22</x:f>
+        <x:v>1000.8333617343287</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="23" customHeight="1">
+      <x:c r="C25" s="132" t="str">
+        <x:v>Closing liquidity after capex savings only</x:v>
+      </x:c>
+      <x:c r="D25" s="149" t="n">
+        <x:f>SUM(D8,D23)</x:f>
+        <x:v>1617.6849384245884</x:v>
+      </x:c>
+      <x:c r="E25" s="149" t="n">
+        <x:f>SUM(E8,E23)</x:f>
+        <x:v>2372.7362520271845</x:v>
+      </x:c>
+      <x:c r="F25" s="149" t="n">
+        <x:f>SUM(F8,F23)</x:f>
+        <x:v>971.8100482292325</x:v>
+      </x:c>
+      <x:c r="G25" s="149" t="n">
+        <x:f>SUM(G8,G23)</x:f>
+        <x:v>499.99999999999955</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="23" customHeight="1">
+      <x:c r="C26" s="158" t="str">
+        <x:v>Cumulative residual funding required</x:v>
+      </x:c>
+      <x:c r="D26" s="159" t="n">
+        <x:f>MAX(0,ROUND(D9-D25,6))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E26" s="159" t="n">
+        <x:f>MAX(D26,ROUND(E9-E25,6))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F26" s="159" t="n">
+        <x:f>MAX(E26,ROUND(F9-F25,6))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G26" s="159" t="n">
+        <x:f>MAX(F26,ROUND(G9-G25,6))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="23" customHeight="1">
+      <x:c r="C27" s="158" t="str">
+        <x:v>Additional residual funding this period</x:v>
+      </x:c>
+      <x:c r="D27" s="159" t="n">
+        <x:f>D26</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="159" t="n">
+        <x:f>E26-D26</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F27" s="159" t="n">
+        <x:f>F26-E26</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G27" s="159" t="n">
+        <x:f>G26-F26</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="23" customHeight="1">
+      <x:c r="C28" s="158" t="str">
+        <x:v>Closing liquidity with cuts and residual funding</x:v>
+      </x:c>
+      <x:c r="D28" s="159" t="n">
+        <x:f>SUM(D25,D26)</x:f>
+        <x:v>1617.6849384245884</x:v>
+      </x:c>
+      <x:c r="E28" s="159" t="n">
+        <x:f>SUM(E25,E26)</x:f>
+        <x:v>2372.7362520271845</x:v>
+      </x:c>
+      <x:c r="F28" s="159" t="n">
+        <x:f>SUM(F25,F26)</x:f>
+        <x:v>971.8100482292325</x:v>
+      </x:c>
+      <x:c r="G28" s="159" t="n">
+        <x:f>SUM(G25,G26)</x:f>
+        <x:v>500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="23" customHeight="1">
+      <x:c r="C29" s="153" t="str">
+        <x:v>Required uniform cut at each liquidity deadline</x:v>
+      </x:c>
+      <x:c r="D29" s="155" t="n">
+        <x:f>IF(D14=0,IF(D10&gt;=0,0,"n.a."),MAX(0,-D10/D14))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E29" s="155" t="n">
+        <x:f>IF(E14=0,IF(E10&gt;=0,0,"n.a."),MAX(0,-E10/E14))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F29" s="155" t="n">
+        <x:f>IF(F14=0,IF(F10&gt;=0,0,"n.a."),MAX(0,-F10/F14))</x:f>
+        <x:v>0.27038202141748635</x:v>
+      </x:c>
+      <x:c r="G29" s="155" t="n">
+        <x:f>IF(G14=0,IF(G10&gt;=0,0,"n.a."),MAX(0,-G10/G14))</x:f>
+        <x:v>0.3327777588437808</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="23" customHeight="1">
+      <x:c r="C30" s="166" t="str">
+        <x:v>HOW TO READ THE TABLE</x:v>
+      </x:c>
+      <x:c r="D30" s="166"/>
+      <x:c r="E30" s="166"/>
+      <x:c r="F30" s="166"/>
+      <x:c r="G30" s="166"/>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="C31" s="165" t="str">
+        <x:v>Alternatives A and B are separate routes. Do not add their funding totals together. Funding amounts are cumulative, not annual sums.</x:v>
+      </x:c>
+      <x:c r="D31" s="165"/>
+      <x:c r="E31" s="165"/>
+      <x:c r="F31" s="165"/>
+      <x:c r="G31" s="165"/>
+    </x:row>
+    <x:row r="32" ht="34" customHeight="1">
+      <x:c r="C32" s="165" t="str">
+        <x:v>Funding is additional to advances, grants/equity and the $100m loan already in Forecast. No extra debt interest, fees or repayments are assumed.</x:v>
+      </x:c>
+      <x:c r="D32" s="165"/>
+      <x:c r="E32" s="165"/>
+      <x:c r="F32" s="165"/>
+      <x:c r="G32" s="165"/>
+    </x:row>
+    <x:row r="33" ht="34" customHeight="1">
+      <x:c r="C33" s="165" t="str">
+        <x:v>Divide each deadline shortfall by capex accumulated to that deadline. The largest ratio is the uniform break-even cut, capped at discretionary spending.</x:v>
+      </x:c>
+      <x:c r="D33" s="165"/>
+      <x:c r="E33" s="165"/>
+      <x:c r="F33" s="165"/>
+      <x:c r="G33" s="165"/>
+    </x:row>
+    <x:row r="34" ht="34" customHeight="1">
+      <x:c r="C34" s="165" t="str">
+        <x:v>Maintenance capex stays at its original estimate. Cuts exceeding discretionary spending leave residual funding. Earlier cuts are assumed to remain available as cash.</x:v>
+      </x:c>
+      <x:c r="D34" s="165"/>
+      <x:c r="E34" s="165"/>
+      <x:c r="F34" s="165"/>
+      <x:c r="G34" s="165"/>
+    </x:row>
+    <x:row r="35" ht="34" customHeight="1">
+      <x:c r="C35" s="165" t="str">
+        <x:v>Savings hold revenue, EBITDA, taxes, working capital, advances/credits and debt service unchanged. This is liquidity arithmetic, not an operating reforecast.</x:v>
+      </x:c>
+      <x:c r="D35" s="165"/>
+      <x:c r="E35" s="165"/>
+      <x:c r="F35" s="165"/>
+      <x:c r="G35" s="165"/>
+    </x:row>
+    <x:row r="36" ht="34" customHeight="1">
+      <x:c r="C36" s="165" t="str">
+        <x:v>Funding/savings must occur before each period-end. Annual/half-year balances do not test daily liquidity. H2 2026 is a full modeled half-year, partly elapsed.</x:v>
+      </x:c>
+      <x:c r="D36" s="165"/>
+      <x:c r="E36" s="165"/>
+      <x:c r="F36" s="165"/>
+      <x:c r="G36" s="165"/>
+    </x:row>
+    <x:row r="37" ht="34" customHeight="1">
+      <x:c r="C37" s="165" t="str">
+        <x:v>Actual capex deferral may require contract/customer consent, reduce advance funding or impair future capacity. Validate timing and consequences before using it.</x:v>
+      </x:c>
+      <x:c r="D37" s="165"/>
+      <x:c r="E37" s="165"/>
+      <x:c r="F37" s="165"/>
+      <x:c r="G37" s="165"/>
+    </x:row>
+    <x:row r="38" ht="34" customHeight="1">
+      <x:c r="C38" s="165" t="str">
+        <x:v>The reserve is an illustrative analyst screen, not an OCBC covenant. Meeting it alone does not establish loan approval or debt-funded repayment capacity.</x:v>
+      </x:c>
+      <x:c r="D38" s="165"/>
+      <x:c r="E38" s="165"/>
+      <x:c r="F38" s="165"/>
+      <x:c r="G38" s="165"/>
+    </x:row>
+    <x:row r="39" ht="23" customHeight="1">
+      <x:c r="C39" s="132"/>
+      <x:c r="D39" s="132"/>
+      <x:c r="E39" s="132"/>
+      <x:c r="F39" s="132"/>
+      <x:c r="G39" s="132"/>
+    </x:row>
+    <x:row r="40" ht="23" customHeight="1">
+      <x:c r="C40" s="132"/>
+      <x:c r="D40" s="132"/>
+      <x:c r="E40" s="132"/>
+      <x:c r="F40" s="132"/>
+      <x:c r="G40" s="132"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="C2:G2"/>
+    <x:mergeCell ref="D4:F4"/>
+    <x:mergeCell ref="C5:G5"/>
+    <x:mergeCell ref="C15:G15"/>
+    <x:mergeCell ref="C20:G20"/>
+    <x:mergeCell ref="D21:G21"/>
+    <x:mergeCell ref="C30:G30"/>
+    <x:mergeCell ref="C31:G31"/>
+    <x:mergeCell ref="C32:G32"/>
+    <x:mergeCell ref="C33:G33"/>
+    <x:mergeCell ref="C34:G34"/>
+    <x:mergeCell ref="C35:G35"/>
+    <x:mergeCell ref="C36:G36"/>
+    <x:mergeCell ref="C37:G37"/>
+    <x:mergeCell ref="C38:G38"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="D10:G10">
+    <x:cfRule type="expression" dxfId="15" priority="1">
+      <x:formula>D10&lt;-0.000001</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="D25:G25">
+    <x:cfRule type="expression" dxfId="16" priority="2">
+      <x:formula>D25&lt;D9-0.000001</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>